<commit_message>
feat: opsi "Tidak Dikreditkan" di impor Pajak Masukan
Kolom PENGKREDITAN PPN pada template Excel sekarang punya pilihan ketiga
"TIDAK DIKREDITKAN" di samping MASA SAMA/MASA TIDAK SAMA - baris dengan
pilihan ini tidak butuh MASA PENGKREDITAN sama sekali dan memanggil
uncreditOne (mesin yang sudah teruji live, sebelumnya belum tersambung
ke jalur impor Excel) alih-alih creditOne. Berlaku juga saat masa
ditetapkan lewat mode "Tetapkan satu masa" di aplikasi - baris yang
ditandai TIDAK DIKREDITKAN tetap tidak dikreditkan meski override aktif.

Update juga sheet PETUNJUK di template dan label nav ("Pengkreditan
Faktur Masukan") + hint di halaman agar mencakup dua arah.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gui/public/assets/template-pajak-masukan.xlsx
+++ b/gui/public/assets/template-pajak-masukan.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="57">
   <si>
     <t>DIISI OLEH ANDA</t>
   </si>
@@ -131,10 +131,10 @@
     <t>Angka polos. Ini yang dipakai sebagai pencocokan utama nilai.</t>
   </si>
   <si>
-    <t>Pilih dari dropdown: MASA SAMA atau MASA TIDAK SAMA. Sel jadi MERAH bila tidak cocok dengan Masa PM vs Masa Pengkreditan.</t>
-  </si>
-  <si>
-    <t>Masa tempat PM dikreditkan. Ketik 01/08/2026, tampil sebagai 08/2026.</t>
+    <t>Pilih dari dropdown: MASA SAMA, MASA TIDAK SAMA, atau TIDAK DIKREDITKAN. Sel jadi MERAH bila tidak cocok dengan Masa PM vs Masa Pengkreditan (aturan ini tidak berlaku untuk TIDAK DIKREDITKAN).</t>
+  </si>
+  <si>
+    <t>Masa tempat PM dikreditkan. Ketik 01/08/2026, tampil sebagai 08/2026. KOSONGKAN bila PENGKREDITAN PPN diisi TIDAK DIKREDITKAN.</t>
   </si>
   <si>
     <t>Aturan yang akan menolak baris Anda</t>
@@ -162,6 +162,12 @@
   </si>
   <si>
     <t>Faktur berstatus CREDITED harus dikembalikan ke APPROVED dulu sebelum masanya bisa diubah.</t>
+  </si>
+  <si>
+    <t>Tidak Dikreditkan</t>
+  </si>
+  <si>
+    <t>Baris dengan PENGKREDITAN PPN = TIDAK DIKREDITKAN mengubah faktur menjadi berstatus Tidak Dikreditkan (bukan dikreditkan ke masa manapun) - kolom MASA PENGKREDITAN diabaikan untuk baris ini.</t>
   </si>
   <si>
     <t>Arti kolom hasil</t>
@@ -5093,11 +5099,11 @@
     <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Harus angka" error="Isi angka tanpa titik/koma pemisah ribuan." sqref="G6:H305">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Pilihan tidak valid" error="Hanya boleh MASA SAMA atau MASA TIDAK SAMA." sqref="I10:I305">
-      <formula1>"MASA SAMA,MASA TIDAK SAMA"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Pilihan tidak valid" error="Hanya boleh MASA SAMA, MASA TIDAK SAMA, atau TIDAK DIKREDITKAN." sqref="I10:I305">
+      <formula1>"MASA SAMA,MASA TIDAK SAMA,TIDAK DIKREDITKAN"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Pilihan tidak valid" error="Hanya boleh MASA SAMA atau MASA TIDAK SAMA." sqref="I6:I305">
-      <formula1>"MASA SAMA,MASA TIDAK SAMA"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Pilihan tidak valid" error="Hanya boleh MASA SAMA, MASA TIDAK SAMA, atau TIDAK DIKREDITKAN." sqref="I6:I305">
+      <formula1>"MASA SAMA,MASA TIDAK SAMA,TIDAK DIKREDITKAN"</formula1>
     </dataValidation>
     <dataValidation type="date" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Masa tidak valid" error="Isi masa pengkreditan, ketik seperti 01/08/2026 (tampil 08/2026)." sqref="J10:J305">
       <formula1>45657.70833333333</formula1>
@@ -5109,13 +5115,13 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:C29"/>
+  <dimension ref="A2:C30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -5269,42 +5275,50 @@
         <v>49</v>
       </c>
     </row>
-    <row r="25" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B25" s="24" t="s">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
         <v>50</v>
       </c>
-      <c r="C25" s="24"/>
-    </row>
-    <row r="26" ht="28" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B26" s="25" t="s">
+      <c r="C24" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B26" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="C26" s="24"/>
+    </row>
+    <row r="27" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B27" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="C26" s="26" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="27" ht="28" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B27" s="25" t="s">
+      <c r="C27" s="26" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="28" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B28" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="C27" s="26" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="28" ht="28" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B28" s="25" t="s">
+      <c r="C28" s="26" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="29" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B29" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="C28" s="26" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="29" ht="28" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B29" s="25" t="s">
+      <c r="C29" s="26" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="30" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B30" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="C29" s="26" t="s">
-        <v>54</v>
+      <c r="C30" s="26" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -5312,9 +5326,9 @@
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: template Pajak Masukan tidak menandai merah baris TIDAK DIKREDITKAN
Aturan format bersyarat kolom PENGKREDITAN PPN membandingkan dengan
MASA SAMA/MASA TIDAK SAMA, jadi baris TIDAK DIKREDITKAN yang MASA
PENGKREDITAN-nya ikut terisi salah tampil merah.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gui/public/assets/template-pajak-masukan.xlsx
+++ b/gui/public/assets/template-pajak-masukan.xlsx
@@ -5065,7 +5065,7 @@
   </mergeCells>
   <conditionalFormatting sqref="I6:I305">
     <cfRule type="expression" dxfId="0" priority="1">
-      <formula>AND($I6&lt;&gt;"",$F6&lt;&gt;"",$J6&lt;&gt;"",IF($F6=$J6,"MASA SAMA","MASA TIDAK SAMA")&lt;&gt;$I6)</formula>
+      <formula>AND($I6&lt;&gt;"",$I6&lt;&gt;"TIDAK DIKREDITKAN",$F6&lt;&gt;"",$J6&lt;&gt;"",IF($F6=$J6,"MASA SAMA","MASA TIDAK SAMA")&lt;&gt;$I6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K6:K305">
@@ -5121,7 +5121,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:C30"/>
+  <dimension ref="B2:C30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -5275,7 +5275,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>50</v>
       </c>
@@ -5283,13 +5283,13 @@
         <v>51</v>
       </c>
     </row>
-    <row r="26" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B26" s="24" t="s">
         <v>52</v>
       </c>
       <c r="C26" s="24"/>
     </row>
-    <row r="27" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" ht="28" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B27" s="25" t="s">
         <v>12</v>
       </c>
@@ -5297,7 +5297,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="28" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" ht="28" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B28" s="25" t="s">
         <v>13</v>
       </c>
@@ -5305,7 +5305,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="29" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" ht="28" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B29" s="25" t="s">
         <v>14</v>
       </c>
@@ -5313,7 +5313,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="30" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" ht="28" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B30" s="25" t="s">
         <v>15</v>
       </c>

</xml_diff>